<commit_message>
Laminas comunales de Migracion, Ocupacion, Pensiones y Salud
Lote 3 de 6.
El commit original (b1bed81b) cambiaba 13.973 archivos y 2,40 GB de objetos
nuevos en una sola pieza. GitHub rechaza los push sobre 2 GB por HTTPS, y SSH
esta bloqueado en esta red, asi que ese commit no podia subir nunca: el HTTP 500
no era un error transitorio sino el limite. Se trocea por dimension, que es un
corte con sentido, no alfabetico.
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_m_saldomigr_a_2019_biobio.xlsx
+++ b/output/graficos_dimensiones/comunal_m_saldomigr_a_2019_biobio.xlsx
@@ -93,12 +93,12 @@
     <t xml:space="preserve">Mulchén</t>
   </si>
   <si>
+    <t xml:space="preserve">Arauco</t>
+  </si>
+  <si>
     <t xml:space="preserve">San Rosendo</t>
   </si>
   <si>
-    <t xml:space="preserve">Arauco</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cañete</t>
   </si>
   <si>
@@ -141,7 +141,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-06 19:40</t>
+    <t xml:space="preserve">2026-09-09 22:26</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -891,7 +891,7 @@
         <v>25</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>8310</v>
+        <v>8202</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>2019</v>
@@ -908,7 +908,7 @@
         <v>26</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>8202</v>
+        <v>8310</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>2019</v>

</xml_diff>